<commit_message>
Setup: pestaña Jira, netlify, gitignore
</commit_message>
<xml_diff>
--- a/Jira_Tickets_GDI.xlsx
+++ b/Jira_Tickets_GDI.xlsx
@@ -8,14 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://intcomexonline-my.sharepoint.com/personal/jpinz390_intcomex_com/Documents/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="39" documentId="11_6472F2DF532DEDA4E07BB6A9AF357AE476D7F4CE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0B7E421-BB72-44AE-ACB9-7EA49069069E}"/>
+  <xr:revisionPtr revIDLastSave="545" documentId="11_6472F2DF532DEDA4E07BB6A9AF357AE476D7F4CE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{369B1C85-84F6-4189-A2FB-42B9CB8A0616}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tickets Jira" sheetId="1" r:id="rId1"/>
-    <sheet name="Instrucciones" sheetId="2" r:id="rId2"/>
+    <sheet name="Hoja1" sheetId="3" r:id="rId2"/>
+    <sheet name="Hoja2" sheetId="4" r:id="rId3"/>
+    <sheet name="Hoja3" sheetId="5" r:id="rId4"/>
+    <sheet name="Instrucciones" sheetId="2" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Hoja2!$B$1:$H$28</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -37,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="137">
   <si>
     <t>Ticket</t>
   </si>
@@ -97,13 +103,364 @@
   </si>
   <si>
     <t>Flujo configurado en: make.powerautomate.com</t>
+  </si>
+  <si>
+    <t>37103-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>37100-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>37079-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>37078-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>37071-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>37058-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>37047-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>37035-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>37034-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>37031-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>37024-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>37009-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>37007-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36992-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36999-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36994-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36989-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36970-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36968-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36932-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36916-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36890-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36852-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36706-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36656-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36626-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36621-CROCS_COL_CCSCOWL180</t>
+  </si>
+  <si>
+    <t>36596-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36597-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36598-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36599-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36600-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36601-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36602-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36603-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36604-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36605-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36606-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36607-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36608-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36609-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36610-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36611-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36612-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36613-CROCS_COL</t>
+  </si>
+  <si>
+    <t>37058-CROCS_COL</t>
+  </si>
+  <si>
+    <t>37071-CROCS_COL</t>
+  </si>
+  <si>
+    <t>37078-CROCS_COL</t>
+  </si>
+  <si>
+    <t>37079-CROCS_COL</t>
+  </si>
+  <si>
+    <t>37103-CROCS_COL</t>
+  </si>
+  <si>
+    <t>37100-CROCS_COL</t>
+  </si>
+  <si>
+    <t>ITHD-94645</t>
+  </si>
+  <si>
+    <t>ITHD-94845</t>
+  </si>
+  <si>
+    <t>Order ID</t>
+  </si>
+  <si>
+    <t>✅</t>
+  </si>
+  <si>
+    <t>❌</t>
+  </si>
+  <si>
+    <t>MPN</t>
+  </si>
+  <si>
+    <t>10001-6ZW-M6W8</t>
+  </si>
+  <si>
+    <t>210581-214-M7W9</t>
+  </si>
+  <si>
+    <t>207989-001-M5W7</t>
+  </si>
+  <si>
+    <t>206991-100-J5</t>
+  </si>
+  <si>
+    <t>210581-214-M8W10</t>
+  </si>
+  <si>
+    <t>211106-90H-M8W10</t>
+  </si>
+  <si>
+    <t>37047-CROCS_COL</t>
+  </si>
+  <si>
+    <t>37035-CROCS_COL</t>
+  </si>
+  <si>
+    <t>37034-CROCS_COL</t>
+  </si>
+  <si>
+    <t>37031-CROCS_COL</t>
+  </si>
+  <si>
+    <t>37024-CROCS_COL</t>
+  </si>
+  <si>
+    <t>37009-CROCS_COL</t>
+  </si>
+  <si>
+    <t>37007-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36999-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36994-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36992-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36989-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36970-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36968-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36932-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36916-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36890-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36852-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36706-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36656-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36626-CROCS_COL</t>
+  </si>
+  <si>
+    <t>36621-CROCS_COL</t>
+  </si>
+  <si>
+    <t>207937-001-M7W9</t>
+  </si>
+  <si>
+    <t>SKU</t>
+  </si>
+  <si>
+    <t>207989-001-M6W8</t>
+  </si>
+  <si>
+    <t>209862-0WW-W8</t>
+  </si>
+  <si>
+    <t>209384-001-W8</t>
+  </si>
+  <si>
+    <t>209401-001-M10W12</t>
+  </si>
+  <si>
+    <t>209964-001-M11</t>
+  </si>
+  <si>
+    <t>209587-5BX-W5</t>
+  </si>
+  <si>
+    <t>207521-2Y2-M4W6</t>
+  </si>
+  <si>
+    <t>10001-4WK-M9W11</t>
+  </si>
+  <si>
+    <t>210989-0WV-C8</t>
+  </si>
+  <si>
+    <t>11016-6UR-M5W7</t>
+  </si>
+  <si>
+    <t>ITHD-94828</t>
+  </si>
+  <si>
+    <t>YPL23CRS31</t>
+  </si>
+  <si>
+    <t>YPL14CRS89</t>
+  </si>
+  <si>
+    <t>YPL09CCS60</t>
+  </si>
+  <si>
+    <t>YPL50CCS60</t>
+  </si>
+  <si>
+    <t>YPL14CRS88</t>
+  </si>
+  <si>
+    <t>YPL17CRS92</t>
+  </si>
+  <si>
+    <t>YPL83CCS03</t>
+  </si>
+  <si>
+    <t>YPL50CCS61</t>
+  </si>
+  <si>
+    <t>YPL91CCS19</t>
+  </si>
+  <si>
+    <t>YPL71CCS98</t>
+  </si>
+  <si>
+    <t>YPL88CCS31</t>
+  </si>
+  <si>
+    <t>YPL16CRS69</t>
+  </si>
+  <si>
+    <t>YPL36CRS14</t>
+  </si>
+  <si>
+    <t>YPL27CCS42</t>
+  </si>
+  <si>
+    <t>YPL21CRS80</t>
+  </si>
+  <si>
+    <t>YPL18CRS40</t>
+  </si>
+  <si>
+    <t>YPL76CCS94</t>
+  </si>
+  <si>
+    <t>Stock en 0</t>
+  </si>
+  <si>
+    <t>Escalado a Kronotime</t>
+  </si>
+  <si>
+    <t>Escalado a CI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -132,8 +489,27 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -150,6 +526,12 @@
         <fgColor rgb="FFF1F5F9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -163,7 +545,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -172,6 +554,16 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -520,7 +912,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="60" customWidth="1"/>
@@ -531,7 +923,7 @@
     <col min="7" max="7" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="27.95" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -554,7 +946,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -586,39 +978,1490 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E15EC15-248F-4CD2-800F-48EEDE38548A}">
+  <dimension ref="B1:G27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="30" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:7">
+      <c r="B1" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="2:7">
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7">
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7">
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7">
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s">
+        <v>68</v>
+      </c>
+      <c r="G5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7">
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7">
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="G7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7">
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" t="s">
+        <v>47</v>
+      </c>
+      <c r="G8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7">
+      <c r="B9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7">
+      <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7">
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" t="s">
+        <v>50</v>
+      </c>
+      <c r="G11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7">
+      <c r="B12" t="s">
+        <v>31</v>
+      </c>
+      <c r="F12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7">
+      <c r="B13" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7">
+      <c r="B14" t="s">
+        <v>33</v>
+      </c>
+      <c r="F14" t="s">
+        <v>53</v>
+      </c>
+      <c r="G14" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7">
+      <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="F15" t="s">
+        <v>54</v>
+      </c>
+      <c r="G15" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7">
+      <c r="B16" t="s">
+        <v>35</v>
+      </c>
+      <c r="F16" t="s">
+        <v>55</v>
+      </c>
+      <c r="G16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7">
+      <c r="B17" t="s">
+        <v>36</v>
+      </c>
+      <c r="F17" t="s">
+        <v>56</v>
+      </c>
+      <c r="G17" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7">
+      <c r="B18" t="s">
+        <v>37</v>
+      </c>
+      <c r="F18" t="s">
+        <v>57</v>
+      </c>
+      <c r="G18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7">
+      <c r="B19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F19" t="s">
+        <v>58</v>
+      </c>
+      <c r="G19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7">
+      <c r="B20" t="s">
+        <v>39</v>
+      </c>
+      <c r="F20" t="s">
+        <v>59</v>
+      </c>
+      <c r="G20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7">
+      <c r="B21" t="s">
+        <v>40</v>
+      </c>
+      <c r="F21" t="s">
+        <v>60</v>
+      </c>
+      <c r="G21" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7">
+      <c r="B22" t="s">
+        <v>41</v>
+      </c>
+      <c r="F22" t="s">
+        <v>61</v>
+      </c>
+      <c r="G22" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7">
+      <c r="B23" t="s">
+        <v>42</v>
+      </c>
+      <c r="F23" t="s">
+        <v>62</v>
+      </c>
+      <c r="G23" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7">
+      <c r="B24" t="s">
+        <v>43</v>
+      </c>
+      <c r="F24" t="s">
+        <v>63</v>
+      </c>
+      <c r="G24" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7">
+      <c r="B25" t="s">
+        <v>44</v>
+      </c>
+      <c r="F25" t="s">
+        <v>64</v>
+      </c>
+      <c r="G25" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7">
+      <c r="B26" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7">
+      <c r="B27" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5765DB7-ED5E-40F7-B0E2-73FE9F7A6AFE}">
+  <sheetPr filterMode="1"/>
+  <dimension ref="B1:J28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="34.28515625" customWidth="1"/>
+    <col min="3" max="4" width="30" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:10">
+      <c r="B1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" t="s">
+        <v>105</v>
+      </c>
+      <c r="D1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="G1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H1" t="s">
+        <v>134</v>
+      </c>
+      <c r="I1" t="s">
+        <v>135</v>
+      </c>
+      <c r="J1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="2:10">
+      <c r="B2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10">
+      <c r="B3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D3" t="s">
+        <v>81</v>
+      </c>
+      <c r="E3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G3" t="s">
+        <v>75</v>
+      </c>
+      <c r="H3" t="s">
+        <v>74</v>
+      </c>
+      <c r="I3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10">
+      <c r="B4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E4" t="s">
+        <v>74</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H4" t="s">
+        <v>74</v>
+      </c>
+      <c r="I4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10">
+      <c r="B5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" t="s">
+        <v>74</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G5" t="s">
+        <v>75</v>
+      </c>
+      <c r="H5" t="s">
+        <v>74</v>
+      </c>
+      <c r="I5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10">
+      <c r="B6" t="s">
+        <v>66</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D6" t="s">
+        <v>78</v>
+      </c>
+      <c r="E6" t="s">
+        <v>74</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G6" t="s">
+        <v>75</v>
+      </c>
+      <c r="H6" t="s">
+        <v>74</v>
+      </c>
+      <c r="I6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10">
+      <c r="B7" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G7" t="s">
+        <v>75</v>
+      </c>
+      <c r="H7" t="s">
+        <v>74</v>
+      </c>
+      <c r="I7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10">
+      <c r="B8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D8" t="s">
+        <v>78</v>
+      </c>
+      <c r="E8" t="s">
+        <v>75</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G8" t="s">
+        <v>75</v>
+      </c>
+      <c r="H8" t="s">
+        <v>74</v>
+      </c>
+      <c r="I8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10">
+      <c r="B9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="D9" t="s">
+        <v>104</v>
+      </c>
+      <c r="E9" t="s">
+        <v>75</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G9" t="s">
+        <v>75</v>
+      </c>
+      <c r="H9" t="s">
+        <v>74</v>
+      </c>
+      <c r="I9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10">
+      <c r="B10" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D10" t="s">
+        <v>81</v>
+      </c>
+      <c r="E10" t="s">
+        <v>75</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G10" t="s">
+        <v>75</v>
+      </c>
+      <c r="H10" t="s">
+        <v>74</v>
+      </c>
+      <c r="I10" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10">
+      <c r="B11" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="D11" t="s">
+        <v>106</v>
+      </c>
+      <c r="E11" t="s">
+        <v>75</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G11" t="s">
+        <v>75</v>
+      </c>
+      <c r="H11" t="s">
+        <v>74</v>
+      </c>
+      <c r="I11" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10">
+      <c r="B12" t="s">
+        <v>87</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D12" t="s">
+        <v>107</v>
+      </c>
+      <c r="E12" t="s">
+        <v>75</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" t="s">
+        <v>75</v>
+      </c>
+      <c r="H12" t="s">
+        <v>74</v>
+      </c>
+      <c r="I12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10">
+      <c r="B13" t="s">
+        <v>88</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="D13" t="s">
+        <v>108</v>
+      </c>
+      <c r="E13" t="s">
+        <v>75</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G13" t="s">
+        <v>75</v>
+      </c>
+      <c r="H13" t="s">
+        <v>74</v>
+      </c>
+      <c r="I13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" hidden="1">
+      <c r="B14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D14" t="s">
+        <v>82</v>
+      </c>
+      <c r="E14" t="s">
+        <v>75</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G14" t="s">
+        <v>75</v>
+      </c>
+      <c r="H14" t="s">
+        <v>75</v>
+      </c>
+      <c r="J14" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" hidden="1">
+      <c r="B15" t="s">
+        <v>90</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D15" t="s">
+        <v>82</v>
+      </c>
+      <c r="E15" t="s">
+        <v>75</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G15" t="s">
+        <v>75</v>
+      </c>
+      <c r="H15" t="s">
+        <v>75</v>
+      </c>
+      <c r="J15" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10">
+      <c r="B16" t="s">
+        <v>91</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D16" t="s">
+        <v>81</v>
+      </c>
+      <c r="E16" t="s">
+        <v>75</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G16" t="s">
+        <v>75</v>
+      </c>
+      <c r="H16" t="s">
+        <v>74</v>
+      </c>
+      <c r="I16" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10">
+      <c r="B17" t="s">
+        <v>92</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="D17" t="s">
+        <v>109</v>
+      </c>
+      <c r="E17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G17" t="s">
+        <v>75</v>
+      </c>
+      <c r="H17" t="s">
+        <v>74</v>
+      </c>
+      <c r="I17" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10">
+      <c r="B18" t="s">
+        <v>93</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="D18" t="s">
+        <v>110</v>
+      </c>
+      <c r="E18" t="s">
+        <v>75</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G18" t="s">
+        <v>75</v>
+      </c>
+      <c r="H18" t="s">
+        <v>74</v>
+      </c>
+      <c r="I18" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10" hidden="1">
+      <c r="B19" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D19" t="s">
+        <v>78</v>
+      </c>
+      <c r="E19" t="s">
+        <v>75</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G19" t="s">
+        <v>75</v>
+      </c>
+      <c r="H19" t="s">
+        <v>75</v>
+      </c>
+      <c r="J19" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" hidden="1">
+      <c r="B20" t="s">
+        <v>95</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D20" t="s">
+        <v>82</v>
+      </c>
+      <c r="E20" t="s">
+        <v>75</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G20" t="s">
+        <v>75</v>
+      </c>
+      <c r="H20" t="s">
+        <v>75</v>
+      </c>
+      <c r="J20" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="2:10">
+      <c r="B21" t="s">
+        <v>96</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D21" t="s">
+        <v>79</v>
+      </c>
+      <c r="E21" t="s">
+        <v>75</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G21" t="s">
+        <v>75</v>
+      </c>
+      <c r="H21" t="s">
+        <v>74</v>
+      </c>
+      <c r="I21" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="2:10" hidden="1">
+      <c r="B22" t="s">
+        <v>97</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D22" t="s">
+        <v>107</v>
+      </c>
+      <c r="E22" t="s">
+        <v>75</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G22" t="s">
+        <v>75</v>
+      </c>
+      <c r="H22" t="s">
+        <v>75</v>
+      </c>
+      <c r="J22" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" spans="2:10">
+      <c r="B23" t="s">
+        <v>98</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="D23" t="s">
+        <v>111</v>
+      </c>
+      <c r="E23" t="s">
+        <v>75</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G23" t="s">
+        <v>75</v>
+      </c>
+      <c r="H23" t="s">
+        <v>74</v>
+      </c>
+      <c r="I23" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="24" spans="2:10">
+      <c r="B24" t="s">
+        <v>99</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="D24" t="s">
+        <v>112</v>
+      </c>
+      <c r="E24" t="s">
+        <v>75</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G24" t="s">
+        <v>75</v>
+      </c>
+      <c r="H24" t="s">
+        <v>74</v>
+      </c>
+      <c r="I24" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="25" spans="2:10">
+      <c r="B25" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="D25" t="s">
+        <v>112</v>
+      </c>
+      <c r="E25" t="s">
+        <v>75</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G25" t="s">
+        <v>75</v>
+      </c>
+      <c r="H25" t="s">
+        <v>74</v>
+      </c>
+      <c r="I25" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="26" spans="2:10">
+      <c r="B26" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="D26" t="s">
+        <v>113</v>
+      </c>
+      <c r="E26" t="s">
+        <v>75</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G26" t="s">
+        <v>75</v>
+      </c>
+      <c r="H26" t="s">
+        <v>74</v>
+      </c>
+      <c r="I26" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="27" spans="2:10" hidden="1">
+      <c r="B27" t="s">
+        <v>102</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D27" t="s">
+        <v>114</v>
+      </c>
+      <c r="E27" t="s">
+        <v>75</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G27" t="s">
+        <v>75</v>
+      </c>
+      <c r="H27" t="s">
+        <v>75</v>
+      </c>
+      <c r="J27" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28" spans="2:10">
+      <c r="B28" t="s">
+        <v>103</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="D28" t="s">
+        <v>115</v>
+      </c>
+      <c r="E28" t="s">
+        <v>75</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G28" t="s">
+        <v>75</v>
+      </c>
+      <c r="H28" t="s">
+        <v>74</v>
+      </c>
+      <c r="I28" t="s">
+        <v>74</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="B1:H28" xr:uid="{B5765DB7-ED5E-40F7-B0E2-73FE9F7A6AFE}">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="✅"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{260F40D7-408C-4ED8-9CED-98059B4BB4CC}">
+  <dimension ref="E7:H34"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="7" spans="5:8">
+      <c r="E7" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="5:8" ht="60">
+      <c r="E8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="5:8" ht="60">
+      <c r="E9" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="5:8" ht="60">
+      <c r="E10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="5:8" ht="60">
+      <c r="E11" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="12" spans="5:8" ht="60">
+      <c r="E12" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="5:8" ht="60">
+      <c r="E13" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" spans="5:8" ht="60">
+      <c r="E14" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="15" spans="5:8" ht="60">
+      <c r="E15" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="5:8" ht="60">
+      <c r="E16" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="5:8" ht="60">
+      <c r="E17" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="5:8" ht="60">
+      <c r="E18" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" spans="5:8" ht="60">
+      <c r="E19" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="5:8" ht="60">
+      <c r="E20" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="5:8" ht="60">
+      <c r="E21" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="5:8" ht="60">
+      <c r="E22" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" spans="5:8" ht="60">
+      <c r="E23" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" spans="5:8" ht="60">
+      <c r="E24" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="5:8" ht="60">
+      <c r="E25" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="5:8" ht="60">
+      <c r="E26" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="5:8" ht="60">
+      <c r="E27" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F27" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="28" spans="5:8" ht="60">
+      <c r="E28" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F28" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="5:8" ht="60">
+      <c r="E29" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="30" spans="5:8" ht="60">
+      <c r="E30" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="31" spans="5:8" ht="60">
+      <c r="E31" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32" spans="5:8" ht="60">
+      <c r="E32" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="33" spans="5:8" ht="60">
+      <c r="E33" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="34" spans="5:8" ht="60">
+      <c r="E34" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F34" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="20.25" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" ht="20.25">
       <c r="A1" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1">
       <c r="A3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1">
       <c r="A4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1">
       <c r="A6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1">
       <c r="A7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1">
       <c r="A9" t="s">
         <v>19</v>
       </c>

</xml_diff>